<commit_message>
Ajoute l'acronyme SAPHO à la liste des acronymes
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/acronymes/acronymes.xlsx
+++ b/data/acronymes/acronymes.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\chu-brest\Public\DIM\Privé\Z_DOCUMENTS\TECH-COD\pmsi_plus\src\data\acronymes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\0159538A\Documents\repo\pmsi-plus\data\acronymes\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1186" uniqueCount="822">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1189" uniqueCount="824">
   <si>
     <t>Abréviation</t>
   </si>
@@ -2554,6 +2554,12 @@
   </si>
   <si>
     <t>bizarre parosteal osteochondromatous proliferation</t>
+  </si>
+  <si>
+    <t>SAPHO</t>
+  </si>
+  <si>
+    <t>Synovitis, Acne, Pustulosis, Hyperostosis and Osteitis : le syndrome SAPHO est considéré comme une maladie rare</t>
   </si>
 </sst>
 </file>
@@ -2826,8 +2832,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tableau1" displayName="Tableau1" ref="A1:C397" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
-  <autoFilter ref="A1:C397"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tableau1" displayName="Tableau1" ref="A1:C398" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
+  <autoFilter ref="A1:C398"/>
   <sortState ref="A8:C402">
     <sortCondition ref="A8"/>
   </sortState>
@@ -3103,7 +3109,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C397"/>
+  <dimension ref="A1:C398"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.140625" style="3" bestFit="1" customWidth="1"/>
@@ -7460,12 +7466,23 @@
     </row>
     <row r="397" spans="1:3" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A397" s="15" t="s">
+        <v>822</v>
+      </c>
+      <c r="B397" s="18" t="s">
+        <v>823</v>
+      </c>
+      <c r="C397" s="5" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="398" spans="1:3" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A398" s="15" t="s">
         <v>820</v>
       </c>
-      <c r="B397" s="16" t="s">
+      <c r="B398" s="16" t="s">
         <v>821</v>
       </c>
-      <c r="C397" s="14" t="s">
+      <c r="C398" s="14" t="s">
         <v>365</v>
       </c>
     </row>

</xml_diff>